<commit_message>
stochatische var is nog niet af
</commit_message>
<xml_diff>
--- a/Maizz.xlsx
+++ b/Maizz.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/milhgjvan/Documents/GitHub/portfolio_compbio_clean/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hvanm\Documents\GitHub\portfolio_compbio_clean\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{003F3227-F05E-5145-8577-44863A3CEA82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0AE34862-629F-4F66-9CA2-3DC073C9C1D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Formulierreacties 1" sheetId="1" r:id="rId1"/>
@@ -376,14 +376,14 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="19.1640625" customWidth="1"/>
-    <col min="5" max="12" width="18.83203125" customWidth="1"/>
+    <col min="1" max="3" width="18.88671875" customWidth="1"/>
+    <col min="4" max="4" width="19.109375" customWidth="1"/>
+    <col min="5" max="12" width="18.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -403,7 +403,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>46269.727988379629</v>
       </c>
@@ -423,7 +423,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>46269.728750381946</v>
       </c>
@@ -449,10 +449,4 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
-<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{d465f887-04a9-4c17-8b62-103eddccf68b}" enabled="1" method="Standard" siteId="{ca2a7f76-dbd7-4ec0-9108-6b3d524fb7c8}" contentBits="0" removed="0"/>
-</clbl:labelList>
 </file>
</xml_diff>